<commit_message>
Add 3 flow channel version. Fix cell thermal separation Fix heat power, cooler recive heat from both sides
</commit_message>
<xml_diff>
--- a/thermal_analysis_results.xlsx
+++ b/thermal_analysis_results.xlsx
@@ -823,13 +823,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D6EC6E5D-D429-49F6-B22A-879562D58739}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C89A2D3A-5244-4384-B988-B2BCCACE6774}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A0A0546F-1FE4-4490-A674-E6DC1C73EF58}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A311D359-4F0B-42F2-9DE6-DBEA74FBBC12}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0985BD66-2A75-47F3-BF83-D72C343EFF2F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B73501B2-1DF7-40E6-A215-ED214B312CE5}"/>
 </file>
</xml_diff>

<commit_message>
Fix values and att wahter glycol valuse
</commit_message>
<xml_diff>
--- a/thermal_analysis_results.xlsx
+++ b/thermal_analysis_results.xlsx
@@ -447,7 +447,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>6.042220282132013</v>
+        <v>11.1698609718881</v>
       </c>
     </row>
     <row r="3">
@@ -457,7 +457,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8.133065844675688</v>
+        <v>13.30091510294224</v>
       </c>
     </row>
     <row r="4">
@@ -467,7 +467,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16.51881007947652</v>
+        <v>16.50604330807044</v>
       </c>
     </row>
     <row r="5">
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32.40731481492841</v>
+        <v>37.92109778288587</v>
       </c>
     </row>
     <row r="6">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>34.49816037747208</v>
+        <v>40.05215191394</v>
       </c>
     </row>
     <row r="7">
@@ -497,7 +497,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>42.88390461227291</v>
+        <v>43.25728011906821</v>
       </c>
     </row>
     <row r="8">
@@ -507,7 +507,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>58.403121942811</v>
+        <v>64.41682427861237</v>
       </c>
     </row>
     <row r="9">
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>60.49396750535468</v>
+        <v>66.5478784096665</v>
       </c>
     </row>
     <row r="10">
@@ -527,7 +527,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>68.87971174015551</v>
+        <v>69.75300661479471</v>
       </c>
     </row>
     <row r="11">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>6.042220282132011</v>
+        <v>11.16986097188811</v>
       </c>
     </row>
     <row r="12">
@@ -547,7 +547,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8.133065844675688</v>
+        <v>13.30091510294223</v>
       </c>
     </row>
     <row r="13">
@@ -557,7 +557,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.51881007947652</v>
+        <v>16.50604330807045</v>
       </c>
     </row>
     <row r="14">
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>25.9958071278826</v>
+        <v>26.49572649572649</v>
       </c>
     </row>
     <row r="15">
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>25.9958071278826</v>
+        <v>26.49572649572649</v>
       </c>
     </row>
     <row r="16">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>25.9958071278826</v>
+        <v>26.4957264957265</v>
       </c>
     </row>
   </sheetData>
@@ -823,13 +823,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C89A2D3A-5244-4384-B988-B2BCCACE6774}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9DEBF10C-4D18-4D1D-A449-56AAE07B45DF}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A311D359-4F0B-42F2-9DE6-DBEA74FBBC12}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A68AEAEA-376B-43E0-8FB7-7FCAA4D9CC8C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B73501B2-1DF7-40E6-A215-ED214B312CE5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{96BDDF06-B535-49B8-AB2D-371F08570C66}"/>
 </file>
</xml_diff>

<commit_message>
Add 1 flow channel simualtions
</commit_message>
<xml_diff>
--- a/thermal_analysis_results.xlsx
+++ b/thermal_analysis_results.xlsx
@@ -823,13 +823,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0106306B-E202-44A2-99ED-7F8235488FD6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{745992C0-C8BC-4ADF-8E92-49478D5B5D14}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CE0A14E6-2E8C-42A0-B7C4-B34761124618}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{32E9C922-C115-44D2-8340-B2E7C3AF936E}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BDB75A41-5D50-4E97-8E9E-9E52E945E16F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5AFE4053-1748-4EA3-9D3A-C342726029D4}"/>
 </file>
</xml_diff>